<commit_message>
Ajout mapping et description d6491f524d3c37c15306abc01fcc866953174449
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-slot-presence-absence.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-slot-presence-absence.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="343">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-12T13:52:17+00:00</t>
+    <t>2026-06-15T09:04:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -658,6 +658,9 @@
   </si>
   <si>
     <t>Indique si une facture a été établie.</t>
+  </si>
+  <si>
+    <t>Statut.statut (pour le statut FACTURE)</t>
   </si>
   <si>
     <t>Slot.modifierExtension</t>
@@ -967,7 +970,7 @@
     <t>Slot.status</t>
   </si>
   <si>
-    <t>busy | free | busy-unavailable | busy-tentative | entered-in-error</t>
+    <t>Correspondance des statuts métier avec les codes FHIR : PLANIFIE → busy-tentative, VALIDE → busy. Le statut FACTURE est couvert par l'extension TDDUIFacturation.</t>
   </si>
   <si>
     <t>busy | free | busy-unavailable | busy-tentative | entered-in-error.</t>
@@ -976,7 +979,7 @@
     <t>http://hl7.org/fhir/ValueSet/slotstatus</t>
   </si>
   <si>
-    <t>Statut.statut</t>
+    <t>Statut.statut (pour les statuts PLANIFIE et VALIDE)</t>
   </si>
   <si>
     <t>FREEBUSY;FBTYPE=(freeBusyType):19980314T233000Z/19980315T003000Z If the freeBusyType is BUSY, then this value can be excluded</t>
@@ -1417,7 +1420,7 @@
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="30.4765625" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="40.49609375" customWidth="true" bestFit="true"/>
     <col min="38" max="38" width="87.9765625" customWidth="true" bestFit="true"/>
     <col min="39" max="39" width="110.453125" customWidth="true" bestFit="true"/>
     <col min="40" max="40" width="31.65234375" customWidth="true" bestFit="true"/>
@@ -3691,7 +3694,7 @@
         <v>116</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>77</v>
+        <v>207</v>
       </c>
       <c r="AL20" t="s" s="2">
         <v>77</v>
@@ -3705,10 +3708,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3734,16 +3737,16 @@
         <v>108</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="N21" t="s" s="2">
         <v>111</v>
       </c>
       <c r="O21" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="P21" t="s" s="2">
         <v>77</v>
@@ -3792,7 +3795,7 @@
         <v>77</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>78</v>
@@ -3821,10 +3824,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3847,13 +3850,13 @@
         <v>89</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3892,7 +3895,7 @@
         <v>77</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AC22" s="2"/>
       <c r="AD22" t="s" s="2">
@@ -3902,7 +3905,7 @@
         <v>114</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>78</v>
@@ -3926,15 +3929,15 @@
         <v>77</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -4043,10 +4046,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4157,10 +4160,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4186,16 +4189,16 @@
         <v>168</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="O25" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>77</v>
@@ -4220,11 +4223,11 @@
         <v>77</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y25" s="2"/>
       <c r="Z25" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>77</v>
@@ -4242,7 +4245,7 @@
         <v>77</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4260,7 +4263,7 @@
         <v>77</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AM25" t="s" s="2">
         <v>77</v>
@@ -4271,10 +4274,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4297,19 +4300,19 @@
         <v>89</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>77</v>
@@ -4337,10 +4340,10 @@
         <v>150</v>
       </c>
       <c r="Y26" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="Z26" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>77</v>
@@ -4358,7 +4361,7 @@
         <v>77</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4376,7 +4379,7 @@
         <v>77</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>77</v>
@@ -4387,10 +4390,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4416,16 +4419,16 @@
         <v>130</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O27" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>77</v>
@@ -4438,7 +4441,7 @@
         <v>77</v>
       </c>
       <c r="T27" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="U27" t="s" s="2">
         <v>77</v>
@@ -4474,7 +4477,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4492,7 +4495,7 @@
         <v>77</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>77</v>
@@ -4503,10 +4506,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4532,13 +4535,13 @@
         <v>102</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4552,7 +4555,7 @@
         <v>77</v>
       </c>
       <c r="T28" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="U28" t="s" s="2">
         <v>77</v>
@@ -4588,7 +4591,7 @@
         <v>77</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4606,7 +4609,7 @@
         <v>77</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AM28" t="s" s="2">
         <v>77</v>
@@ -4617,10 +4620,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4643,13 +4646,13 @@
         <v>89</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4700,7 +4703,7 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -4718,7 +4721,7 @@
         <v>77</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>77</v>
@@ -4729,10 +4732,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4755,16 +4758,16 @@
         <v>89</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4814,7 +4817,7 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4832,7 +4835,7 @@
         <v>77</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>77</v>
@@ -4843,13 +4846,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D31" t="s" s="2">
         <v>77</v>
@@ -4871,13 +4874,13 @@
         <v>89</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
@@ -4928,7 +4931,7 @@
         <v>77</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -4940,10 +4943,10 @@
         <v>77</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>77</v>
@@ -4952,15 +4955,15 @@
         <v>77</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5069,10 +5072,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5183,10 +5186,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5212,16 +5215,16 @@
         <v>168</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>77</v>
@@ -5246,11 +5249,11 @@
         <v>77</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y34" s="2"/>
       <c r="Z34" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>77</v>
@@ -5268,7 +5271,7 @@
         <v>77</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5286,7 +5289,7 @@
         <v>77</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AM34" t="s" s="2">
         <v>77</v>
@@ -5297,10 +5300,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5323,19 +5326,19 @@
         <v>89</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>77</v>
@@ -5345,7 +5348,7 @@
         <v>77</v>
       </c>
       <c r="S35" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="T35" t="s" s="2">
         <v>77</v>
@@ -5363,10 +5366,10 @@
         <v>150</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>77</v>
@@ -5384,7 +5387,7 @@
         <v>77</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5402,7 +5405,7 @@
         <v>77</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AM35" t="s" s="2">
         <v>77</v>
@@ -5413,10 +5416,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5442,16 +5445,16 @@
         <v>130</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>77</v>
@@ -5461,10 +5464,10 @@
         <v>77</v>
       </c>
       <c r="S36" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="T36" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="U36" t="s" s="2">
         <v>77</v>
@@ -5500,7 +5503,7 @@
         <v>77</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5518,7 +5521,7 @@
         <v>77</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="AM36" t="s" s="2">
         <v>77</v>
@@ -5529,10 +5532,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5558,13 +5561,13 @@
         <v>102</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5578,7 +5581,7 @@
         <v>77</v>
       </c>
       <c r="T37" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="U37" t="s" s="2">
         <v>77</v>
@@ -5614,7 +5617,7 @@
         <v>77</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -5632,7 +5635,7 @@
         <v>77</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>77</v>
@@ -5643,10 +5646,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5669,13 +5672,13 @@
         <v>89</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5726,7 +5729,7 @@
         <v>77</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -5744,7 +5747,7 @@
         <v>77</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="AM38" t="s" s="2">
         <v>77</v>
@@ -5755,10 +5758,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5781,16 +5784,16 @@
         <v>89</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
@@ -5840,7 +5843,7 @@
         <v>77</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -5858,7 +5861,7 @@
         <v>77</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="AM39" t="s" s="2">
         <v>77</v>
@@ -5869,10 +5872,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5895,13 +5898,13 @@
         <v>89</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5932,7 +5935,7 @@
       </c>
       <c r="Y40" s="2"/>
       <c r="Z40" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>77</v>
@@ -5950,7 +5953,7 @@
         <v>77</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -5974,15 +5977,15 @@
         <v>77</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6005,13 +6008,13 @@
         <v>89</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6038,11 +6041,11 @@
         <v>77</v>
       </c>
       <c r="X41" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y41" s="2"/>
       <c r="Z41" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>77</v>
@@ -6060,7 +6063,7 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6075,7 +6078,7 @@
         <v>100</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="AL41" t="s" s="2">
         <v>77</v>
@@ -6084,15 +6087,15 @@
         <v>77</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6115,13 +6118,13 @@
         <v>89</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6148,11 +6151,11 @@
         <v>77</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y42" s="2"/>
       <c r="Z42" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>77</v>
@@ -6170,7 +6173,7 @@
         <v>77</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6194,15 +6197,15 @@
         <v>77</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6225,13 +6228,13 @@
         <v>89</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6258,11 +6261,11 @@
         <v>77</v>
       </c>
       <c r="X43" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y43" s="2"/>
       <c r="Z43" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>77</v>
@@ -6280,7 +6283,7 @@
         <v>77</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6295,7 +6298,7 @@
         <v>100</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AL43" t="s" s="2">
         <v>77</v>
@@ -6304,15 +6307,15 @@
         <v>77</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6335,13 +6338,13 @@
         <v>89</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6392,7 +6395,7 @@
         <v>77</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>88</v>
@@ -6421,10 +6424,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6450,10 +6453,10 @@
         <v>168</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6480,11 +6483,11 @@
         <v>77</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y45" s="2"/>
       <c r="Z45" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>77</v>
@@ -6502,7 +6505,7 @@
         <v>77</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>88</v>
@@ -6517,13 +6520,13 @@
         <v>100</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM45" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>77</v>
@@ -6531,10 +6534,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6560,10 +6563,10 @@
         <v>102</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -6643,10 +6646,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6753,13 +6756,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="B48" t="s" s="2">
         <v>314</v>
       </c>
-      <c r="B48" t="s" s="2">
-        <v>313</v>
-      </c>
       <c r="C48" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D48" t="s" s="2">
         <v>77</v>
@@ -6781,13 +6784,13 @@
         <v>77</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -6853,7 +6856,7 @@
         <v>116</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>77</v>
@@ -6867,10 +6870,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6896,10 +6899,10 @@
         <v>102</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -6950,7 +6953,7 @@
         <v>77</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -6979,10 +6982,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7008,10 +7011,10 @@
         <v>123</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7062,7 +7065,7 @@
         <v>77</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>88</v>
@@ -7077,24 +7080,24 @@
         <v>100</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="AL50" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM50" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="AN50" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7120,10 +7123,10 @@
         <v>123</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7174,7 +7177,7 @@
         <v>77</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>88</v>
@@ -7189,24 +7192,24 @@
         <v>100</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AL51" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AM51" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="AN51" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7229,13 +7232,13 @@
         <v>77</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -7243,7 +7246,7 @@
         <v>77</v>
       </c>
       <c r="Q52" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="R52" t="s" s="2">
         <v>77</v>
@@ -7288,7 +7291,7 @@
         <v>77</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>78</v>
@@ -7317,10 +7320,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7346,10 +7349,10 @@
         <v>102</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7400,7 +7403,7 @@
         <v>77</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>

</xml_diff>

<commit_message>
Ajout règle de gestion absencePrevueCardinality, correction motifAbsenceCardinality et modification des exemeples fc97b8ecbeeb0f51cfc988885eb2b7f71cc725a2
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-slot-presence-absence.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-slot-presence-absence.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-15T09:04:15+00:00</t>
+    <t>2026-06-16T10:03:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -266,7 +266,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}motifAbsenceCardinality:Cet attribut est obligatoire pour les typePresenceAbsence=Absence {(serviceType.coding.code='2') implies (appointmentType.exists())}absencePrevueCardinality:Cet attribut est obligatoire pour les typePresenceAbsence=Absence {(serviceType.coding.code='2') implies (extension[TDDUIPlannedAbsence].exists())}</t>
   </si>
   <si>
     <t>PresenceAbsence</t>

</xml_diff>

<commit_message>
Update de la description des invariants et ajout du binding pour les identifier 1276a621407ea853b55534a8c702caa7a2000105
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-slot-presence-absence.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-slot-presence-absence.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1926" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="342">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-16T13:10:49+00:00</t>
+    <t>2026-06-22T08:40:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -266,7 +266,7 @@
   </si>
   <si>
     <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}motifAbsenceCardinality:Cet attribut est obligatoire pour les typePresenceAbsence=Absence {(serviceType.coding.code='2') implies (appointmentType.exists())}absencePrevueCardinality:Cet attribut est obligatoire pour les typePresenceAbsence=Absence {(serviceType.coding.code='2') implies (extension.where(url = 'https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-planned-absence').exists())}</t>
+dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}motifAbsenceCardinality:motifAbsence est obligatoire pour les typePresenceAbsence=Absence {(serviceType.coding.code='2') implies (appointmentType.exists())}absencePrevueCardinality:absencePrevue est obligatoire pour les typePresenceAbsence=Absence {(serviceType.coding.code='2') implies (extension.where(url = 'https://interop.esante.gouv.fr/ig/fhir/tddui/StructureDefinition/tddui-planned-absence').exists())}</t>
   </si>
   <si>
     <t>PresenceAbsence</t>
@@ -751,10 +751,7 @@
     <t>Allows users to make use of identifiers when the identifier system is not known.</t>
   </si>
   <si>
-    <t>A coded type for an identifier that can be used to determine which identifier to use for a specific purpose.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/identifier-type</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/tddui/ValueSet/tddui-slot-identifier-presence-absence</t>
   </si>
   <si>
     <t>Identifier.type</t>
@@ -1410,7 +1407,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="84.54296875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="60.9453125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="71.83984375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
@@ -4337,31 +4334,29 @@
         <v>77</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="Y26" t="s" s="2">
+        <v>226</v>
+      </c>
+      <c r="Y26" s="2"/>
+      <c r="Z26" t="s" s="2">
         <v>236</v>
       </c>
-      <c r="Z26" t="s" s="2">
+      <c r="AA26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF26" t="s" s="2">
         <v>237</v>
-      </c>
-      <c r="AA26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE26" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF26" t="s" s="2">
-        <v>238</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4390,10 +4385,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4419,16 +4414,16 @@
         <v>130</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="M27" t="s" s="2">
+      <c r="N27" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="N27" t="s" s="2">
+      <c r="O27" t="s" s="2">
         <v>242</v>
-      </c>
-      <c r="O27" t="s" s="2">
-        <v>243</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>77</v>
@@ -4441,43 +4436,43 @@
         <v>77</v>
       </c>
       <c r="T27" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="U27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF27" t="s" s="2">
         <v>244</v>
-      </c>
-      <c r="U27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE27" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF27" t="s" s="2">
-        <v>245</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4495,7 +4490,7 @@
         <v>77</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>77</v>
@@ -4506,10 +4501,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4535,13 +4530,13 @@
         <v>102</v>
       </c>
       <c r="L28" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="M28" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="M28" t="s" s="2">
+      <c r="N28" t="s" s="2">
         <v>249</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>250</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -4555,43 +4550,43 @@
         <v>77</v>
       </c>
       <c r="T28" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="U28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE28" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF28" t="s" s="2">
         <v>251</v>
-      </c>
-      <c r="U28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF28" t="s" s="2">
-        <v>252</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4609,7 +4604,7 @@
         <v>77</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="AM28" t="s" s="2">
         <v>77</v>
@@ -4620,10 +4615,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4646,13 +4641,13 @@
         <v>89</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>255</v>
       </c>
-      <c r="L29" t="s" s="2">
+      <c r="M29" t="s" s="2">
         <v>256</v>
-      </c>
-      <c r="M29" t="s" s="2">
-        <v>257</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4703,7 +4698,7 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -4721,7 +4716,7 @@
         <v>77</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>77</v>
@@ -4732,10 +4727,10 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4758,16 +4753,16 @@
         <v>89</v>
       </c>
       <c r="K30" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="L30" t="s" s="2">
         <v>261</v>
       </c>
-      <c r="L30" t="s" s="2">
+      <c r="M30" t="s" s="2">
         <v>262</v>
       </c>
-      <c r="M30" t="s" s="2">
+      <c r="N30" t="s" s="2">
         <v>263</v>
-      </c>
-      <c r="N30" t="s" s="2">
-        <v>264</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4817,7 +4812,7 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4835,7 +4830,7 @@
         <v>77</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>77</v>
@@ -4846,13 +4841,13 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B31" t="s" s="2">
         <v>213</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D31" t="s" s="2">
         <v>77</v>
@@ -4877,7 +4872,7 @@
         <v>214</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="M31" t="s" s="2">
         <v>216</v>
@@ -4943,10 +4938,10 @@
         <v>77</v>
       </c>
       <c r="AJ31" t="s" s="2">
+        <v>269</v>
+      </c>
+      <c r="AK31" t="s" s="2">
         <v>270</v>
-      </c>
-      <c r="AK31" t="s" s="2">
-        <v>271</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>77</v>
@@ -4960,7 +4955,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B32" t="s" s="2">
         <v>219</v>
@@ -5072,7 +5067,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B33" t="s" s="2">
         <v>220</v>
@@ -5186,7 +5181,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B34" t="s" s="2">
         <v>221</v>
@@ -5300,7 +5295,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B35" t="s" s="2">
         <v>230</v>
@@ -5348,7 +5343,7 @@
         <v>77</v>
       </c>
       <c r="S35" t="s" s="2">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="T35" t="s" s="2">
         <v>77</v>
@@ -5363,31 +5358,29 @@
         <v>77</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="Y35" t="s" s="2">
+        <v>226</v>
+      </c>
+      <c r="Y35" s="2"/>
+      <c r="Z35" t="s" s="2">
         <v>236</v>
       </c>
-      <c r="Z35" t="s" s="2">
+      <c r="AA35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE35" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF35" t="s" s="2">
         <v>237</v>
-      </c>
-      <c r="AA35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF35" t="s" s="2">
-        <v>238</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5416,10 +5409,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5445,16 +5438,16 @@
         <v>130</v>
       </c>
       <c r="L36" t="s" s="2">
+        <v>239</v>
+      </c>
+      <c r="M36" t="s" s="2">
         <v>240</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="N36" t="s" s="2">
         <v>241</v>
       </c>
-      <c r="N36" t="s" s="2">
+      <c r="O36" t="s" s="2">
         <v>242</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>243</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>77</v>
@@ -5464,46 +5457,46 @@
         <v>77</v>
       </c>
       <c r="S36" t="s" s="2">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="T36" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="U36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE36" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF36" t="s" s="2">
         <v>244</v>
-      </c>
-      <c r="U36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE36" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF36" t="s" s="2">
-        <v>245</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5521,7 +5514,7 @@
         <v>77</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="AM36" t="s" s="2">
         <v>77</v>
@@ -5532,10 +5525,10 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5561,13 +5554,13 @@
         <v>102</v>
       </c>
       <c r="L37" t="s" s="2">
+        <v>247</v>
+      </c>
+      <c r="M37" t="s" s="2">
         <v>248</v>
       </c>
-      <c r="M37" t="s" s="2">
+      <c r="N37" t="s" s="2">
         <v>249</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>250</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5581,43 +5574,43 @@
         <v>77</v>
       </c>
       <c r="T37" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="U37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE37" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF37" t="s" s="2">
         <v>251</v>
-      </c>
-      <c r="U37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE37" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF37" t="s" s="2">
-        <v>252</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -5635,7 +5628,7 @@
         <v>77</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>77</v>
@@ -5646,10 +5639,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5672,13 +5665,13 @@
         <v>89</v>
       </c>
       <c r="K38" t="s" s="2">
+        <v>254</v>
+      </c>
+      <c r="L38" t="s" s="2">
         <v>255</v>
       </c>
-      <c r="L38" t="s" s="2">
+      <c r="M38" t="s" s="2">
         <v>256</v>
-      </c>
-      <c r="M38" t="s" s="2">
-        <v>257</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5729,7 +5722,7 @@
         <v>77</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -5747,7 +5740,7 @@
         <v>77</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="AM38" t="s" s="2">
         <v>77</v>
@@ -5758,10 +5751,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5784,16 +5777,16 @@
         <v>89</v>
       </c>
       <c r="K39" t="s" s="2">
+        <v>260</v>
+      </c>
+      <c r="L39" t="s" s="2">
         <v>261</v>
       </c>
-      <c r="L39" t="s" s="2">
+      <c r="M39" t="s" s="2">
         <v>262</v>
       </c>
-      <c r="M39" t="s" s="2">
+      <c r="N39" t="s" s="2">
         <v>263</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>264</v>
       </c>
       <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
@@ -5843,7 +5836,7 @@
         <v>77</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -5861,7 +5854,7 @@
         <v>77</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="AM39" t="s" s="2">
         <v>77</v>
@@ -5872,10 +5865,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5901,10 +5894,10 @@
         <v>231</v>
       </c>
       <c r="L40" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="M40" t="s" s="2">
         <v>283</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>284</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5935,7 +5928,7 @@
       </c>
       <c r="Y40" s="2"/>
       <c r="Z40" t="s" s="2">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>77</v>
@@ -5953,7 +5946,7 @@
         <v>77</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
@@ -5977,15 +5970,15 @@
         <v>77</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6011,10 +6004,10 @@
         <v>231</v>
       </c>
       <c r="L41" t="s" s="2">
+        <v>287</v>
+      </c>
+      <c r="M41" t="s" s="2">
         <v>288</v>
-      </c>
-      <c r="M41" t="s" s="2">
-        <v>289</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6045,7 +6038,7 @@
       </c>
       <c r="Y41" s="2"/>
       <c r="Z41" t="s" s="2">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>77</v>
@@ -6063,7 +6056,7 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
@@ -6078,7 +6071,7 @@
         <v>100</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="AL41" t="s" s="2">
         <v>77</v>
@@ -6087,15 +6080,15 @@
         <v>77</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6121,10 +6114,10 @@
         <v>231</v>
       </c>
       <c r="L42" t="s" s="2">
+        <v>292</v>
+      </c>
+      <c r="M42" t="s" s="2">
         <v>293</v>
-      </c>
-      <c r="M42" t="s" s="2">
-        <v>294</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6155,7 +6148,7 @@
       </c>
       <c r="Y42" s="2"/>
       <c r="Z42" t="s" s="2">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>77</v>
@@ -6173,7 +6166,7 @@
         <v>77</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>78</v>
@@ -6197,15 +6190,15 @@
         <v>77</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6231,10 +6224,10 @@
         <v>231</v>
       </c>
       <c r="L43" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>297</v>
-      </c>
-      <c r="M43" t="s" s="2">
-        <v>298</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -6265,7 +6258,7 @@
       </c>
       <c r="Y43" s="2"/>
       <c r="Z43" t="s" s="2">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="AA43" t="s" s="2">
         <v>77</v>
@@ -6283,7 +6276,7 @@
         <v>77</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
@@ -6298,7 +6291,7 @@
         <v>100</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AL43" t="s" s="2">
         <v>77</v>
@@ -6307,15 +6300,15 @@
         <v>77</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6338,13 +6331,13 @@
         <v>89</v>
       </c>
       <c r="K44" t="s" s="2">
+        <v>301</v>
+      </c>
+      <c r="L44" t="s" s="2">
         <v>302</v>
       </c>
-      <c r="L44" t="s" s="2">
+      <c r="M44" t="s" s="2">
         <v>303</v>
-      </c>
-      <c r="M44" t="s" s="2">
-        <v>304</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6395,7 +6388,7 @@
         <v>77</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>88</v>
@@ -6424,10 +6417,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6453,10 +6446,10 @@
         <v>168</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>305</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>306</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>307</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6487,7 +6480,7 @@
       </c>
       <c r="Y45" s="2"/>
       <c r="Z45" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>77</v>
@@ -6505,7 +6498,7 @@
         <v>77</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>88</v>
@@ -6520,13 +6513,13 @@
         <v>100</v>
       </c>
       <c r="AK45" t="s" s="2">
+        <v>308</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM45" t="s" s="2">
         <v>309</v>
-      </c>
-      <c r="AL45" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AM45" t="s" s="2">
-        <v>310</v>
       </c>
       <c r="AN45" t="s" s="2">
         <v>77</v>
@@ -6534,10 +6527,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6563,10 +6556,10 @@
         <v>102</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>311</v>
+      </c>
+      <c r="M46" t="s" s="2">
         <v>312</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>313</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -6646,10 +6639,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6756,13 +6749,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
+        <v>314</v>
+      </c>
+      <c r="B48" t="s" s="2">
+        <v>313</v>
+      </c>
+      <c r="C48" t="s" s="2">
         <v>315</v>
-      </c>
-      <c r="B48" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="C48" t="s" s="2">
-        <v>316</v>
       </c>
       <c r="D48" t="s" s="2">
         <v>77</v>
@@ -6784,13 +6777,13 @@
         <v>77</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>316</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>317</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="M48" t="s" s="2">
         <v>318</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>319</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -6856,7 +6849,7 @@
         <v>116</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>77</v>
@@ -6870,10 +6863,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -6899,10 +6892,10 @@
         <v>102</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -6953,7 +6946,7 @@
         <v>77</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>78</v>
@@ -6982,10 +6975,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7011,10 +7004,10 @@
         <v>123</v>
       </c>
       <c r="L50" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>325</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>326</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7065,7 +7058,7 @@
         <v>77</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>88</v>
@@ -7080,24 +7073,24 @@
         <v>100</v>
       </c>
       <c r="AK50" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="AL50" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM50" t="s" s="2">
         <v>327</v>
       </c>
-      <c r="AL50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AM50" t="s" s="2">
+      <c r="AN50" t="s" s="2">
         <v>328</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>329</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7123,10 +7116,10 @@
         <v>123</v>
       </c>
       <c r="L51" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="M51" t="s" s="2">
         <v>331</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>332</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7177,7 +7170,7 @@
         <v>77</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>88</v>
@@ -7192,24 +7185,24 @@
         <v>100</v>
       </c>
       <c r="AK51" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="AL51" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AM51" t="s" s="2">
         <v>333</v>
       </c>
-      <c r="AL51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AM51" t="s" s="2">
-        <v>334</v>
-      </c>
       <c r="AN51" t="s" s="2">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7232,13 +7225,13 @@
         <v>77</v>
       </c>
       <c r="K52" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="L52" t="s" s="2">
         <v>336</v>
       </c>
-      <c r="L52" t="s" s="2">
+      <c r="M52" t="s" s="2">
         <v>337</v>
-      </c>
-      <c r="M52" t="s" s="2">
-        <v>338</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -7246,7 +7239,7 @@
         <v>77</v>
       </c>
       <c r="Q52" t="s" s="2">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="R52" t="s" s="2">
         <v>77</v>
@@ -7291,7 +7284,7 @@
         <v>77</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>78</v>
@@ -7320,10 +7313,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7349,10 +7342,10 @@
         <v>102</v>
       </c>
       <c r="L53" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="M53" t="s" s="2">
         <v>341</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>342</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7403,7 +7396,7 @@
         <v>77</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>78</v>

</xml_diff>